<commit_message>
Fixing a bug caused by wreckless behaviour... oups
</commit_message>
<xml_diff>
--- a/crate_data.xlsx
+++ b/crate_data.xlsx
@@ -459,28 +459,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Wooden</t>
+          <t>Type A</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>872.85</v>
+        <v>802.5</v>
       </c>
       <c r="D2" t="n">
-        <v>819.0700000000001</v>
+        <v>738.75</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>148x110x259</t>
+          <t>161x111x234</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>7cdff39f-6e66-42da-9664-d4208d5232d1</t>
+          <t>3fff6e08-d50d-4692-abfd-c54fa7ff6274</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
     </row>
@@ -490,28 +490,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Type A</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>880.99</v>
+        <v>867.67</v>
       </c>
       <c r="D3" t="n">
-        <v>792.28</v>
+        <v>773.0599999999999</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>131x124x255</t>
+          <t>161x108x247</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>270fc2e6-4433-4439-b612-8fc5e67d3f4f</t>
+          <t>f3c69746-43ca-48c1-8a83-cdf6f294a3b4</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R10</t>
         </is>
       </c>
     </row>
@@ -521,23 +521,23 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Plastic</t>
+          <t>Type D</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>825.9400000000001</v>
+        <v>803.1799999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>743.79</v>
+        <v>748.5</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>148x110x257</t>
+          <t>161x111x234</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>9f3ae04b-a026-4cc9-8675-00b76428d236</t>
+          <t>eb3642eb-4507-406c-b3f8-c76554826628</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -552,28 +552,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Type A</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>867.16</v>
+        <v>856.12</v>
       </c>
       <c r="D5" t="n">
-        <v>777.47</v>
+        <v>770.3200000000001</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>165x115x259</t>
+          <t>154x131x257</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>28126ccb-c374-4d09-aa9d-b8837228ce37</t>
+          <t>89e688bb-5c7c-4435-9404-6a2ddf8d1cd2</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R7</t>
         </is>
       </c>
     </row>
@@ -583,28 +583,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Wooden</t>
+          <t>Type B</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>896.12</v>
+        <v>844.92</v>
       </c>
       <c r="D6" t="n">
-        <v>816.54</v>
+        <v>781.01</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>140x107x250</t>
+          <t>141x107x234</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>be8ce229-e331-46f0-83a6-6451b1be77f1</t>
+          <t>5e953233-35a9-46d5-b365-4aa078a71aa1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>R3</t>
         </is>
       </c>
     </row>
@@ -614,28 +614,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Type D</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>811.67</v>
+        <v>834.03</v>
       </c>
       <c r="D7" t="n">
-        <v>721.28</v>
+        <v>776.26</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>161x101x251</t>
+          <t>155x115x234</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>db7ffe16-6890-4048-b1b0-05a9c8f4a3c1</t>
+          <t>0fe2145b-f048-4fad-8b8c-1e9c9a8069c6</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
     </row>
@@ -645,28 +645,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Type A</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>822.5700000000001</v>
+        <v>837.99</v>
       </c>
       <c r="D8" t="n">
-        <v>765.5</v>
+        <v>770.04</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>121x117x254</t>
+          <t>155x115x234</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1cb2203d-e5cd-4691-ae12-1f4231cacb41</t>
+          <t>4520ab7f-5fae-4e1b-b332-b283ac69ecd8</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R10</t>
         </is>
       </c>
     </row>
@@ -676,23 +676,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Wooden</t>
+          <t>Type C</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>827.64</v>
+        <v>880.71</v>
       </c>
       <c r="D9" t="n">
-        <v>754.54</v>
+        <v>794.22</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>113x122x256</t>
+          <t>154x131x257</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>c600a988-9a2d-448d-bd62-e1f0ff4c6a8c</t>
+          <t>0e0d3752-5ad9-46eb-8a87-003d02ddd74c</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -707,28 +707,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Plastic</t>
+          <t>Type D</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>841.1</v>
+        <v>807.88</v>
       </c>
       <c r="D10" t="n">
-        <v>769.47</v>
+        <v>743.22</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>155x124x253</t>
+          <t>151x120x232</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>e2b7e0bf-b694-4183-aea1-56d3057d9884</t>
+          <t>c2f21401-e7fc-4282-af39-74a98d21c606</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R10</t>
         </is>
       </c>
     </row>
@@ -738,28 +738,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Plastic</t>
+          <t>Type C</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>843.47</v>
+        <v>857.74</v>
       </c>
       <c r="D11" t="n">
-        <v>752.51</v>
+        <v>772.51</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>148x111x250</t>
+          <t>141x107x234</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>71b40a9f-377e-4d7d-80c8-9fe346dd3a80</t>
+          <t>5f678bd5-2d2d-49b6-98c3-df6350cf87b5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R4</t>
         </is>
       </c>
     </row>
@@ -769,28 +769,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Plastic</t>
+          <t>Type C</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>844.09</v>
+        <v>898.52</v>
       </c>
       <c r="D12" t="n">
-        <v>773.63</v>
+        <v>805.75</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>145x116x259</t>
+          <t>161x108x247</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>c7ea2dab-261d-49c2-b5ff-2e0e37ae9ac6</t>
+          <t>b6e043d2-42e3-4b32-acb5-5028f54b6e1f</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R7</t>
         </is>
       </c>
     </row>
@@ -800,28 +800,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Wooden</t>
+          <t>Type C</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>882.7</v>
+        <v>845.34</v>
       </c>
       <c r="D13" t="n">
-        <v>830.3</v>
+        <v>753.63</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>161x116x251</t>
+          <t>142x115x259</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>02b93974-98eb-4235-b1f1-0559c4cb6a9d</t>
+          <t>08d98cfb-a35e-4205-9877-b04be2ec7700</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R6</t>
         </is>
       </c>
     </row>
@@ -831,28 +831,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Plastic</t>
+          <t>Type C</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>883.02</v>
+        <v>820.95</v>
       </c>
       <c r="D14" t="n">
-        <v>790.39</v>
+        <v>757.6</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>136x121x254</t>
+          <t>151x120x232</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>73dd0d18-0b2f-423d-87f5-ab1df318cba5</t>
+          <t>c5ea12bf-45ed-4149-9e91-4c84080ee8fd</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R2</t>
         </is>
       </c>
     </row>
@@ -862,28 +862,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Type B</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>869.29</v>
+        <v>853.41</v>
       </c>
       <c r="D15" t="n">
-        <v>801.89</v>
+        <v>791.17</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>147x122x251</t>
+          <t>147x131x257</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ee62470a-eac3-49b8-a2ff-a863d97ff628</t>
+          <t>65a77e54-b36d-4799-9e71-d6c984f3ff15</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R7</t>
         </is>
       </c>
     </row>
@@ -893,28 +893,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Plastic</t>
+          <t>Type C</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>812.4299999999999</v>
+        <v>898.95</v>
       </c>
       <c r="D16" t="n">
-        <v>751.3</v>
+        <v>816.95</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>151x102x258</t>
+          <t>154x131x257</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>9e21b2db-a351-4dba-a89a-0b5e48f29e58</t>
+          <t>4ab5b9ba-93b9-4173-83b5-fc271bce5880</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R4</t>
         </is>
       </c>
     </row>
@@ -924,23 +924,23 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Wooden</t>
+          <t>Type C</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>808.7</v>
+        <v>884.29</v>
       </c>
       <c r="D17" t="n">
-        <v>733.36</v>
+        <v>795.49</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>153x125x259</t>
+          <t>161x111x234</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>a2427aea-b47f-4a66-b904-665f65ebbe58</t>
+          <t>024a3a07-3871-468c-882c-cb2e4856bde9</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -955,28 +955,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Plastic</t>
+          <t>Type C</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>874.7</v>
+        <v>840.12</v>
       </c>
       <c r="D18" t="n">
-        <v>810.24</v>
+        <v>786.8099999999999</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>152x125x255</t>
+          <t>145x131x231</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>885243fc-74d2-4979-a92e-e7c1b52a4070</t>
+          <t>4f502514-25af-48f7-8427-9abed36d41a6</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>R10</t>
+          <t>R6</t>
         </is>
       </c>
     </row>
@@ -986,28 +986,28 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Wooden</t>
+          <t>Type B</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>808.95</v>
+        <v>865.54</v>
       </c>
       <c r="D19" t="n">
-        <v>747.41</v>
+        <v>795.76</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>164x112x251</t>
+          <t>151x120x232</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>87f99c48-24b4-4088-957a-9e6525bf849e</t>
+          <t>acc66f72-800a-4923-93c6-ea9f57a77f36</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R8</t>
         </is>
       </c>
     </row>
@@ -1017,28 +1017,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Wooden</t>
+          <t>Type B</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>803.5599999999999</v>
+        <v>826.49</v>
       </c>
       <c r="D20" t="n">
-        <v>744.5599999999999</v>
+        <v>764.16</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>155x110x251</t>
+          <t>154x131x257</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>d4524b5e-38bf-4e12-8102-125f9270203f</t>
+          <t>d54647e3-0e7f-4abe-a404-94cecfa759c2</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R9</t>
         </is>
       </c>
     </row>
@@ -1048,28 +1048,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Type C</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>813.64</v>
+        <v>874.7</v>
       </c>
       <c r="D21" t="n">
-        <v>728.15</v>
+        <v>803.28</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>156x121x257</t>
+          <t>145x131x231</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2eb303b7-48bf-440d-a33b-443a3bf7ec2b</t>
+          <t>7ad07a55-84e0-400d-b916-6a6512284ce0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R7</t>
         </is>
       </c>
     </row>
@@ -1079,28 +1079,28 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Plastic</t>
+          <t>Type C</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>806.23</v>
+        <v>821.9299999999999</v>
       </c>
       <c r="D22" t="n">
-        <v>715.33</v>
+        <v>722.05</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>112x108x256</t>
+          <t>154x131x257</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>8b5f8fb8-ecac-444c-b2c4-61040d8d4a5b</t>
+          <t>3e3dc344-b154-49ba-8f92-bd667580ec67</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R8</t>
         </is>
       </c>
     </row>
@@ -1110,28 +1110,28 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Type A</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>865.92</v>
+        <v>875.58</v>
       </c>
       <c r="D23" t="n">
-        <v>774.42</v>
+        <v>782.52</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>140x112x251</t>
+          <t>142x115x259</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>42f0e0e2-0cc3-4a87-b267-6382bf5d8faa</t>
+          <t>d58ff637-9f66-4d7f-8802-f878acac4d92</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R3</t>
         </is>
       </c>
     </row>
@@ -1141,28 +1141,28 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Type D</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>884.15</v>
+        <v>859.64</v>
       </c>
       <c r="D24" t="n">
-        <v>813.66</v>
+        <v>790.4</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>154x120x253</t>
+          <t>145x131x231</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>127f23d9-d174-4f27-b5a8-7345d71f39a9</t>
+          <t>e68d917a-5b6b-468d-b379-f8681f67f964</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>R10</t>
+          <t>R8</t>
         </is>
       </c>
     </row>
@@ -1172,28 +1172,28 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Wooden</t>
+          <t>Type C</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>852.48</v>
+        <v>897.11</v>
       </c>
       <c r="D25" t="n">
-        <v>799.36</v>
+        <v>804.0700000000001</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>148x106x259</t>
+          <t>141x107x234</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>e83171e8-9ffd-4b54-a78e-d9e6801558f7</t>
+          <t>87d1aec2-6689-4584-9fe5-1e594cf407cd</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R2</t>
         </is>
       </c>
     </row>
@@ -1203,28 +1203,28 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Plastic</t>
+          <t>Type C</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>843.96</v>
+        <v>876.86</v>
       </c>
       <c r="D26" t="n">
-        <v>785.76</v>
+        <v>809.85</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>159x122x255</t>
+          <t>151x131x257</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>4723d397-7b0f-4a02-99d1-58070b1e47a8</t>
+          <t>cc72a3de-95f6-44a6-88ec-1f92427211ae</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R7</t>
         </is>
       </c>
     </row>

</xml_diff>